<commit_message>
vault backup: 2026-10-05 21:47:57
</commit_message>
<xml_diff>
--- a/11_名古屋/A01_薬の履歴.xlsx
+++ b/11_名古屋/A01_薬の履歴.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -59,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -68,6 +72,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -441,6 +449,8 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,6 +479,16 @@
           <t>2026/07/24（21日分）</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2026/08/04（30mL）</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2026/08/25（40g）</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -481,6 +501,16 @@
           <t>かわな病院 吉川先生</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>かわな病院 吉川先生（皮膚科）</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>かわな病院 吉川先生（皮膚科）</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -634,6 +664,64 @@
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>キシロカインゼリー2%</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>適量</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>右脚のキズ（処置前）</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>処置の15〜30分前に塗布</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>カデックス軟膏0.9%</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>1日1回</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>右脚のキズ（床ずれ・皮膚潰瘍）</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>★床ずれや皮膚潰瘍等に用いる</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>○</t>
         </is>

</xml_diff>